<commit_message>
Fix Excel number formatting: percentage columns use plain number format instead of 0.00% (which multiplied by 100)
</commit_message>
<xml_diff>
--- a/Results/strategy_results.xlsx
+++ b/Results/strategy_results.xlsx
@@ -176,7 +176,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -186,21 +186,21 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="9" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="9" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>

</xml_diff>